<commit_message>
Add versioned 178A execution profiles
</commit_message>
<xml_diff>
--- a/cases/_templates/178A/config.xlsx
+++ b/cases/_templates/178A/config.xlsx
@@ -577,7 +577,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F146"/>
+  <dimension ref="A1:F145"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.453125" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" style="11" min="1" max="1"/>
@@ -595,6 +595,14 @@
       </c>
       <c r="F1" s="31" t="n"/>
     </row>
+    <row r="2">
+      <c r="A2" s="12" t="n"/>
+      <c r="B2" s="12" t="n"/>
+      <c r="C2" s="12" t="n"/>
+      <c r="D2" s="12" t="n"/>
+      <c r="E2" s="12" t="n"/>
+      <c r="F2" s="12" t="n"/>
+    </row>
     <row r="3" ht="15" customHeight="1" s="13">
       <c r="A3" s="42" t="inlineStr">
         <is>
@@ -638,7 +646,7 @@
           <t>case_id</t>
         </is>
       </c>
-      <c r="C4" s="26" t="str"/>
+      <c r="C4" s="26" t="n"/>
       <c r="D4" s="35" t="n"/>
       <c r="E4" s="44" t="inlineStr">
         <is>
@@ -662,7 +670,7 @@
           <t>source_config</t>
         </is>
       </c>
-      <c r="C5" s="26" t="str"/>
+      <c r="C5" s="26" t="n"/>
       <c r="D5" s="35" t="n"/>
       <c r="E5" s="44" t="inlineStr">
         <is>
@@ -686,7 +694,7 @@
           <t>source_note</t>
         </is>
       </c>
-      <c r="C6" s="26" t="str"/>
+      <c r="C6" s="26" t="n"/>
       <c r="D6" s="35" t="n"/>
       <c r="E6" s="44" t="inlineStr">
         <is>
@@ -4588,63 +4596,14 @@
       </c>
     </row>
     <row r="145" s="13">
-      <c r="A145" s="39" t="inlineStr">
-        <is>
-          <t>reference</t>
-        </is>
-      </c>
-      <c r="B145" s="39" t="inlineStr">
-        <is>
-          <t>align_to_ref</t>
-        </is>
-      </c>
-      <c r="C145" s="26" t="inlineStr">
-        <is>
-          <t>policy</t>
-        </is>
-      </c>
-      <c r="D145" s="39" t="b">
-        <v>0</v>
-      </c>
-      <c r="E145" s="39" t="inlineStr">
-        <is>
-          <t>bool</t>
-        </is>
-      </c>
-      <c r="F145" s="39" t="inlineStr">
-        <is>
-          <t>Enable the pinned SiCoPR/COM MATLAB 4.17 comparison profile for 178A.</t>
-        </is>
-      </c>
-    </row>
-    <row r="146" s="13">
-      <c r="A146" s="39" t="inlineStr">
-        <is>
-          <t>reference</t>
-        </is>
-      </c>
-      <c r="B146" s="39" t="inlineStr">
-        <is>
-          <t>noise_grid_num_ui</t>
-        </is>
-      </c>
-      <c r="C146" s="26" t="inlineStr">
-        <is>
-          <t>policy</t>
-        </is>
-      </c>
-      <c r="D146" s="39" t="n"/>
-      <c r="E146" s="39" t="inlineStr">
-        <is>
-          <t>UI</t>
-        </is>
-      </c>
-      <c r="F146" s="39" t="inlineStr">
-        <is>
-          <t>MMSE noise PSD/correlation record length; blank uses the analysis grid. The reference preset defaults to 4096 UI.</t>
-        </is>
-      </c>
-    </row>
+      <c r="A145" s="39" t="n"/>
+      <c r="B145" s="39" t="n"/>
+      <c r="C145" s="26" t="n"/>
+      <c r="D145" s="39" t="n"/>
+      <c r="E145" s="39" t="n"/>
+      <c r="F145" s="39" t="n"/>
+    </row>
+    <row r="146" s="13"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:E1"/>
@@ -5160,7 +5119,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E29"/>
+  <dimension ref="A1:E30"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.453125" defaultRowHeight="15"/>
   <cols>
     <col width="13.02999973297119" customWidth="1" style="16" min="1" max="1"/>
@@ -5207,27 +5166,27 @@
     <row r="4" ht="15" customHeight="1" s="13">
       <c r="A4" s="20" t="inlineStr">
         <is>
-          <t>single_run</t>
+          <t>control</t>
         </is>
       </c>
       <c r="B4" s="20" t="inlineStr">
         <is>
-          <t>target</t>
+          <t>execution_profile</t>
         </is>
       </c>
       <c r="C4" s="20" t="inlineStr">
         <is>
-          <t>dfe</t>
+          <t>project_standard</t>
         </is>
       </c>
       <c r="D4" s="20" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>enum</t>
         </is>
       </c>
       <c r="E4" s="20" t="inlineStr">
         <is>
-          <t>Full single-run target.</t>
+          <t>Execution profile: project_standard, sicopr_reference_v1, or custom.</t>
         </is>
       </c>
     </row>
@@ -5239,12 +5198,12 @@
       </c>
       <c r="B5" s="20" t="inlineStr">
         <is>
-          <t>pre_dte_pmf_method</t>
+          <t>target</t>
         </is>
       </c>
       <c r="C5" s="20" t="inlineStr">
         <is>
-          <t>pmf_exact</t>
+          <t>dfe</t>
         </is>
       </c>
       <c r="D5" s="20" t="inlineStr">
@@ -5254,7 +5213,7 @@
       </c>
       <c r="E5" s="20" t="inlineStr">
         <is>
-          <t>Pre-DTE ADC PMF method for V_qc.</t>
+          <t>Full single-run target.</t>
         </is>
       </c>
     </row>
@@ -5266,12 +5225,12 @@
       </c>
       <c r="B6" s="20" t="inlineStr">
         <is>
-          <t>pmf_grid_quality</t>
+          <t>pre_dte_pmf_method</t>
         </is>
       </c>
       <c r="C6" s="20" t="inlineStr">
         <is>
-          <t>coarse</t>
+          <t>pmf_exact</t>
         </is>
       </c>
       <c r="D6" s="20" t="inlineStr">
@@ -5281,7 +5240,7 @@
       </c>
       <c r="E6" s="20" t="inlineStr">
         <is>
-          <t>PMF amplitude-grid quality.</t>
+          <t>Pre-DTE ADC PMF method for V_qc.</t>
         </is>
       </c>
     </row>
@@ -5293,20 +5252,22 @@
       </c>
       <c r="B7" s="20" t="inlineStr">
         <is>
-          <t>pmf_keep_mass</t>
-        </is>
-      </c>
-      <c r="C7" s="20" t="n">
-        <v>0.99999</v>
+          <t>pmf_grid_quality</t>
+        </is>
+      </c>
+      <c r="C7" s="20" t="inlineStr">
+        <is>
+          <t>coarse</t>
+        </is>
       </c>
       <c r="D7" s="20" t="inlineStr">
         <is>
-          <t>probability</t>
+          <t>text</t>
         </is>
       </c>
       <c r="E7" s="20" t="inlineStr">
         <is>
-          <t>Execution-policy PMF mass retained after each ADC-input convolution; final COM overrides this to 1.0.</t>
+          <t>PMF amplitude-grid quality.</t>
         </is>
       </c>
     </row>
@@ -5318,22 +5279,20 @@
       </c>
       <c r="B8" s="20" t="inlineStr">
         <is>
-          <t>floating_mode</t>
-        </is>
-      </c>
-      <c r="C8" s="20" t="inlineStr">
-        <is>
-          <t>spec-defined</t>
-        </is>
+          <t>pmf_keep_mass</t>
+        </is>
+      </c>
+      <c r="C8" s="20" t="n">
+        <v>0.99999</v>
       </c>
       <c r="D8" s="20" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>probability</t>
         </is>
       </c>
       <c r="E8" s="20" t="inlineStr">
         <is>
-          <t>FFE floating-group selection.</t>
+          <t>Execution-policy PMF mass retained after each ADC-input convolution; final COM overrides this to 1.0.</t>
         </is>
       </c>
     </row>
@@ -5345,12 +5304,12 @@
       </c>
       <c r="B9" s="20" t="inlineStr">
         <is>
-          <t>pos_sweep_method</t>
+          <t>floating_mode</t>
         </is>
       </c>
       <c r="C9" s="20" t="inlineStr">
         <is>
-          <t>each_phase</t>
+          <t>spec-defined</t>
         </is>
       </c>
       <c r="D9" s="20" t="inlineStr">
@@ -5360,7 +5319,7 @@
       </c>
       <c r="E9" s="20" t="inlineStr">
         <is>
-          <t>Sampling-phase sweep strategy.</t>
+          <t>FFE floating-group selection.</t>
         </is>
       </c>
     </row>
@@ -5372,47 +5331,47 @@
       </c>
       <c r="B10" s="20" t="inlineStr">
         <is>
-          <t>pos_coarse_stride</t>
-        </is>
-      </c>
-      <c r="C10" s="20" t="n">
-        <v>4</v>
+          <t>pos_sweep_method</t>
+        </is>
+      </c>
+      <c r="C10" s="20" t="inlineStr">
+        <is>
+          <t>each_phase</t>
+        </is>
       </c>
       <c r="D10" s="20" t="inlineStr">
         <is>
-          <t>phase index</t>
+          <t>text</t>
         </is>
       </c>
       <c r="E10" s="20" t="inlineStr">
         <is>
-          <t>Coarse phase stride; used only by coarse_fine.</t>
+          <t>Sampling-phase sweep strategy.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="15" customHeight="1" s="13">
       <c r="A11" s="20" t="inlineStr">
         <is>
-          <t>search_sweep</t>
+          <t>single_run</t>
         </is>
       </c>
       <c r="B11" s="20" t="inlineStr">
         <is>
-          <t>target</t>
-        </is>
-      </c>
-      <c r="C11" s="20" t="inlineStr">
-        <is>
-          <t>mse</t>
-        </is>
+          <t>pos_coarse_stride</t>
+        </is>
+      </c>
+      <c r="C11" s="20" t="n">
+        <v>4</v>
       </c>
       <c r="D11" s="20" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>phase index</t>
         </is>
       </c>
       <c r="E11" s="20" t="inlineStr">
         <is>
-          <t>Partial-search candidate evaluation target.</t>
+          <t>Coarse phase stride; used only by coarse_fine.</t>
         </is>
       </c>
     </row>
@@ -5424,12 +5383,12 @@
       </c>
       <c r="B12" s="20" t="inlineStr">
         <is>
-          <t>pre_dte_pmf_method</t>
+          <t>target</t>
         </is>
       </c>
       <c r="C12" s="20" t="inlineStr">
         <is>
-          <t>pmf_exact</t>
+          <t>mse</t>
         </is>
       </c>
       <c r="D12" s="20" t="inlineStr">
@@ -5439,7 +5398,7 @@
       </c>
       <c r="E12" s="20" t="inlineStr">
         <is>
-          <t>Pre-DTE ADC PMF method for V_qc.</t>
+          <t>Partial-search candidate evaluation target.</t>
         </is>
       </c>
     </row>
@@ -5451,12 +5410,12 @@
       </c>
       <c r="B13" s="20" t="inlineStr">
         <is>
-          <t>pmf_grid_quality</t>
+          <t>pre_dte_pmf_method</t>
         </is>
       </c>
       <c r="C13" s="20" t="inlineStr">
         <is>
-          <t>coarse</t>
+          <t>pmf_exact</t>
         </is>
       </c>
       <c r="D13" s="20" t="inlineStr">
@@ -5466,7 +5425,7 @@
       </c>
       <c r="E13" s="20" t="inlineStr">
         <is>
-          <t>PMF amplitude-grid quality.</t>
+          <t>Pre-DTE ADC PMF method for V_qc.</t>
         </is>
       </c>
     </row>
@@ -5478,20 +5437,22 @@
       </c>
       <c r="B14" s="20" t="inlineStr">
         <is>
-          <t>pmf_keep_mass</t>
-        </is>
-      </c>
-      <c r="C14" s="20" t="n">
-        <v>0.99999</v>
+          <t>pmf_grid_quality</t>
+        </is>
+      </c>
+      <c r="C14" s="20" t="inlineStr">
+        <is>
+          <t>coarse</t>
+        </is>
       </c>
       <c r="D14" s="20" t="inlineStr">
         <is>
-          <t>probability</t>
+          <t>text</t>
         </is>
       </c>
       <c r="E14" s="20" t="inlineStr">
         <is>
-          <t>Execution-policy PMF mass retained after each ADC-input convolution; final COM overrides this to 1.0.</t>
+          <t>PMF amplitude-grid quality.</t>
         </is>
       </c>
     </row>
@@ -5503,22 +5464,20 @@
       </c>
       <c r="B15" s="20" t="inlineStr">
         <is>
-          <t>floating_mode</t>
-        </is>
-      </c>
-      <c r="C15" s="11" t="inlineStr">
-        <is>
-          <t>simplified</t>
-        </is>
+          <t>pmf_keep_mass</t>
+        </is>
+      </c>
+      <c r="C15" s="11" t="n">
+        <v>0.99999</v>
       </c>
       <c r="D15" s="20" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>probability</t>
         </is>
       </c>
       <c r="E15" s="20" t="inlineStr">
         <is>
-          <t>FFE floating-group selection.</t>
+          <t>Execution-policy PMF mass retained after each ADC-input convolution; final COM overrides this to 1.0.</t>
         </is>
       </c>
     </row>
@@ -5530,12 +5489,12 @@
       </c>
       <c r="B16" s="20" t="inlineStr">
         <is>
-          <t>pos_sweep_method</t>
+          <t>floating_mode</t>
         </is>
       </c>
       <c r="C16" s="11" t="inlineStr">
         <is>
-          <t>coarse_fine</t>
+          <t>simplified</t>
         </is>
       </c>
       <c r="D16" s="20" t="inlineStr">
@@ -5545,7 +5504,7 @@
       </c>
       <c r="E16" s="20" t="inlineStr">
         <is>
-          <t>Sampling-phase sweep strategy.</t>
+          <t>FFE floating-group selection.</t>
         </is>
       </c>
     </row>
@@ -5557,47 +5516,47 @@
       </c>
       <c r="B17" s="22" t="inlineStr">
         <is>
-          <t>pos_coarse_stride</t>
-        </is>
-      </c>
-      <c r="C17" s="22" t="n">
-        <v>4</v>
+          <t>pos_sweep_method</t>
+        </is>
+      </c>
+      <c r="C17" s="22" t="inlineStr">
+        <is>
+          <t>coarse_fine</t>
+        </is>
       </c>
       <c r="D17" s="22" t="inlineStr">
         <is>
-          <t>phase index</t>
+          <t>text</t>
         </is>
       </c>
       <c r="E17" s="22" t="inlineStr">
         <is>
-          <t>Coarse phase stride; used only by coarse_fine.</t>
+          <t>Sampling-phase sweep strategy.</t>
         </is>
       </c>
     </row>
     <row r="18" ht="15" customHeight="1" s="13">
       <c r="A18" s="22" t="inlineStr">
         <is>
-          <t>search_final</t>
+          <t>search_sweep</t>
         </is>
       </c>
       <c r="B18" s="22" t="inlineStr">
         <is>
-          <t>target</t>
-        </is>
-      </c>
-      <c r="C18" s="22" t="inlineStr">
-        <is>
-          <t>dfe</t>
-        </is>
+          <t>pos_coarse_stride</t>
+        </is>
+      </c>
+      <c r="C18" s="22" t="n">
+        <v>4</v>
       </c>
       <c r="D18" s="22" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>phase index</t>
         </is>
       </c>
       <c r="E18" s="22" t="inlineStr">
         <is>
-          <t>Top-K final evaluation target.</t>
+          <t>Coarse phase stride; used only by coarse_fine.</t>
         </is>
       </c>
     </row>
@@ -5609,12 +5568,12 @@
       </c>
       <c r="B19" s="22" t="inlineStr">
         <is>
-          <t>pre_dte_pmf_method</t>
+          <t>target</t>
         </is>
       </c>
       <c r="C19" s="22" t="inlineStr">
         <is>
-          <t>pmf_exact</t>
+          <t>dfe</t>
         </is>
       </c>
       <c r="D19" s="22" t="inlineStr">
@@ -5624,7 +5583,7 @@
       </c>
       <c r="E19" s="22" t="inlineStr">
         <is>
-          <t>Pre-DTE ADC PMF method for V_qc.</t>
+          <t>Top-K final evaluation target.</t>
         </is>
       </c>
     </row>
@@ -5636,12 +5595,12 @@
       </c>
       <c r="B20" s="22" t="inlineStr">
         <is>
-          <t>pmf_grid_quality</t>
+          <t>pre_dte_pmf_method</t>
         </is>
       </c>
       <c r="C20" s="22" t="inlineStr">
         <is>
-          <t>coarse</t>
+          <t>pmf_exact</t>
         </is>
       </c>
       <c r="D20" s="22" t="inlineStr">
@@ -5651,7 +5610,7 @@
       </c>
       <c r="E20" s="22" t="inlineStr">
         <is>
-          <t>PMF amplitude-grid quality.</t>
+          <t>Pre-DTE ADC PMF method for V_qc.</t>
         </is>
       </c>
     </row>
@@ -5663,20 +5622,22 @@
       </c>
       <c r="B21" s="22" t="inlineStr">
         <is>
-          <t>pmf_keep_mass</t>
-        </is>
-      </c>
-      <c r="C21" s="22" t="n">
-        <v>0.99999</v>
+          <t>pmf_grid_quality</t>
+        </is>
+      </c>
+      <c r="C21" s="22" t="inlineStr">
+        <is>
+          <t>coarse</t>
+        </is>
       </c>
       <c r="D21" s="22" t="inlineStr">
         <is>
-          <t>probability</t>
+          <t>text</t>
         </is>
       </c>
       <c r="E21" s="22" t="inlineStr">
         <is>
-          <t>Execution-policy PMF mass retained after each ADC-input convolution; final COM overrides this to 1.0.</t>
+          <t>PMF amplitude-grid quality.</t>
         </is>
       </c>
     </row>
@@ -5688,22 +5649,20 @@
       </c>
       <c r="B22" s="22" t="inlineStr">
         <is>
-          <t>floating_mode</t>
-        </is>
-      </c>
-      <c r="C22" s="22" t="inlineStr">
-        <is>
-          <t>spec-defined</t>
-        </is>
+          <t>pmf_keep_mass</t>
+        </is>
+      </c>
+      <c r="C22" s="22" t="n">
+        <v>0.99999</v>
       </c>
       <c r="D22" s="22" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>probability</t>
         </is>
       </c>
       <c r="E22" s="22" t="inlineStr">
         <is>
-          <t>FFE floating-group selection.</t>
+          <t>Execution-policy PMF mass retained after each ADC-input convolution; final COM overrides this to 1.0.</t>
         </is>
       </c>
     </row>
@@ -5715,12 +5674,12 @@
       </c>
       <c r="B23" s="22" t="inlineStr">
         <is>
-          <t>pos_sweep_method</t>
+          <t>floating_mode</t>
         </is>
       </c>
       <c r="C23" s="22" t="inlineStr">
         <is>
-          <t>each_phase</t>
+          <t>spec-defined</t>
         </is>
       </c>
       <c r="D23" s="22" t="inlineStr">
@@ -5730,7 +5689,7 @@
       </c>
       <c r="E23" s="22" t="inlineStr">
         <is>
-          <t>Sampling-phase sweep strategy.</t>
+          <t>FFE floating-group selection.</t>
         </is>
       </c>
     </row>
@@ -5742,45 +5701,47 @@
       </c>
       <c r="B24" s="22" t="inlineStr">
         <is>
-          <t>pos_coarse_stride</t>
-        </is>
-      </c>
-      <c r="C24" s="22" t="n">
-        <v>4</v>
+          <t>pos_sweep_method</t>
+        </is>
+      </c>
+      <c r="C24" s="22" t="inlineStr">
+        <is>
+          <t>each_phase</t>
+        </is>
       </c>
       <c r="D24" s="22" t="inlineStr">
         <is>
-          <t>phase index</t>
+          <t>text</t>
         </is>
       </c>
       <c r="E24" s="22" t="inlineStr">
         <is>
-          <t>Coarse phase stride; used only by coarse_fine.</t>
+          <t>Sampling-phase sweep strategy.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="22" t="inlineStr">
         <is>
-          <t>search</t>
+          <t>search_final</t>
         </is>
       </c>
       <c r="B25" s="22" t="inlineStr">
         <is>
-          <t>group_size</t>
+          <t>pos_coarse_stride</t>
         </is>
       </c>
       <c r="C25" s="16" t="n">
-        <v>100</v>
+        <v>4</v>
       </c>
       <c r="D25" s="22" t="inlineStr">
         <is>
-          <t>count</t>
+          <t>phase index</t>
         </is>
       </c>
       <c r="E25" s="22" t="inlineStr">
         <is>
-          <t>Manifest candidates per partial-search group.</t>
+          <t>Coarse phase stride; used only by coarse_fine.</t>
         </is>
       </c>
     </row>
@@ -5792,11 +5753,11 @@
       </c>
       <c r="B26" s="22" t="inlineStr">
         <is>
-          <t>top_k</t>
+          <t>group_size</t>
         </is>
       </c>
       <c r="C26" s="16" t="n">
-        <v>10</v>
+        <v>100</v>
       </c>
       <c r="D26" s="22" t="inlineStr">
         <is>
@@ -5805,37 +5766,39 @@
       </c>
       <c r="E26" s="22" t="inlineStr">
         <is>
-          <t>Minimum-MSE candidates re-evaluated by search_final.</t>
+          <t>Manifest candidates per partial-search group.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="20" t="inlineStr">
         <is>
-          <t>single_run</t>
+          <t>search</t>
         </is>
       </c>
       <c r="B27" s="20" t="inlineStr">
         <is>
-          <t>pmf_dy_override</t>
-        </is>
-      </c>
-      <c r="C27" s="20" t="n"/>
+          <t>top_k</t>
+        </is>
+      </c>
+      <c r="C27" s="20" t="n">
+        <v>10</v>
+      </c>
       <c r="D27" s="20" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>count</t>
         </is>
       </c>
       <c r="E27" s="20" t="inlineStr">
         <is>
-          <t>Optional direct PMF dy for this run profile; overrides relative/absolute grid derivation.</t>
+          <t>Minimum-MSE candidates re-evaluated by search_final.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="20" t="inlineStr">
         <is>
-          <t>search_sweep</t>
+          <t>single_run</t>
         </is>
       </c>
       <c r="B28" s="20" t="inlineStr">
@@ -5858,7 +5821,7 @@
     <row r="29">
       <c r="A29" s="22" t="inlineStr">
         <is>
-          <t>search_final</t>
+          <t>search_sweep</t>
         </is>
       </c>
       <c r="B29" s="22" t="inlineStr">
@@ -5873,6 +5836,29 @@
         </is>
       </c>
       <c r="E29" s="22" t="inlineStr">
+        <is>
+          <t>Optional direct PMF dy for this run profile; overrides relative/absolute grid derivation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="12" t="inlineStr">
+        <is>
+          <t>search_final</t>
+        </is>
+      </c>
+      <c r="B30" s="12" t="inlineStr">
+        <is>
+          <t>pmf_dy_override</t>
+        </is>
+      </c>
+      <c r="C30" s="12" t="n"/>
+      <c r="D30" s="12" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="E30" s="12" t="inlineStr">
         <is>
           <t>Optional direct PMF dy for this run profile; overrides relative/absolute grid derivation.</t>
         </is>
@@ -5883,9 +5869,8 @@
     <mergeCell ref="A1:E1"/>
   </mergeCells>
   <dataValidations count="18">
-    <dataValidation sqref="C4" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list" errorStyle="stop" operator="between">
-      <formula1>"mse,dfe,mlsd,full"</formula1>
-      <formula2>0</formula2>
+    <dataValidation sqref="C4" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list" errorStyle="stop">
+      <formula1>"project_standard,sicopr_reference_v1,custom"</formula1>
     </dataValidation>
     <dataValidation sqref="C5" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list" errorStyle="stop" operator="between">
       <formula1>"gaussian_approx,pmf_exact"</formula1>

</xml_diff>